<commit_message>
Updated chart widget and added edit budget functionality
</commit_message>
<xml_diff>
--- a/src/utils/sample-budget-3.xlsx
+++ b/src/utils/sample-budget-3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/T.Kellum/Development/budgeteer/src/utils/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D6090F8-BC29-2448-9244-0B3D6031E278}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3704A593-5FD8-AC46-B947-53417E474121}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="80" yWindow="500" windowWidth="25440" windowHeight="14360" activeTab="1" xr2:uid="{3492D7F7-60B5-E14D-B1FF-47B1329F285D}"/>
   </bookViews>
@@ -137,7 +137,28 @@
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -470,9 +491,17 @@
   <dimension ref="A1:AM123"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11" bestFit="1" customWidth="1"/>
     <col min="27" max="27" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="11.1640625" bestFit="1" customWidth="1"/>
   </cols>
@@ -5301,7 +5330,9 @@
   <dimension ref="A5:E502"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.1640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" bestFit="1" customWidth="1"/>
   </cols>
@@ -12801,6 +12832,12 @@
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A6:C502">
     <sortCondition ref="A6:A502"/>
   </sortState>
+  <conditionalFormatting sqref="D6:D502">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>